<commit_message>
Admin: edit data/shala-team.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/shala-team.xlsx
+++ b/data/shala-team.xlsx
@@ -418,10 +418,10 @@
         <v>Shweta Chaudhari</v>
       </c>
       <c r="B2" t="str">
-        <v>Shala Principal</v>
+        <v xml:space="preserve"> Principal</v>
       </c>
       <c r="C2" t="str">
-        <v xml:space="preserve"> Management</v>
+        <v xml:space="preserve"> Shala Management</v>
       </c>
       <c r="D2" t="str">
         <v>assets/images/team/shweta-chaudhari.jpg</v>

</xml_diff>